<commit_message>
fix(planilla): la planilla de asistencia usa las siglas del sistema F FJ T TJ
La planilla manual (PDF y Excel) usaba la leyenda del SIAGIE F J T U, distinta
de la del sistema desde la asistencia por fechas, y su J chocaba con la J de
jueves en la cabecera de dias.

- PlanillaAsistenciaModel::LEYENDA pasa a F/FJ/T/TJ y es el punto unico: el PDF
  la lee directo y generarExcel() escribe desde ella los encabezados de totales
  y la leyenda del pie.
- La plantilla lleva vacias AC8:AF8 y A46 (con su estilo): XlsxQuirurgico no
  sobrescribe celdas con valor, a proposito.
- verif_rol_auxiliar.php: asertos de las siglas nuevas y de la leyenda unica.
- verif_direccion_solo_lectura.php entiende los if partidos en varias lineas;
  daba un falso positivo en matriculas/show.php (el bloque sigue bajo
  $puedeGestionar). Probadas las dos ramas.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/resources/plantillas/registro-asistencia.xlsx
+++ b/resources/plantillas/registro-asistencia.xlsx
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="20">
   <si>
     <t>UNIVERSIDAD NACIONAL SANTIAGO ANTÚNEZ DE MAYOLO</t>
   </si>
@@ -1482,18 +1482,10 @@
       <c r="Z8" s="29"/>
       <c r="AA8" s="29"/>
       <c r="AB8" s="56"/>
-      <c r="AC8" s="62" t="s">
-        <v>10</v>
-      </c>
-      <c r="AD8" s="30" t="s">
-        <v>11</v>
-      </c>
-      <c r="AE8" s="30" t="s">
-        <v>12</v>
-      </c>
-      <c r="AF8" s="71" t="s">
-        <v>13</v>
-      </c>
+      <c r="AC8" s="62"/>
+      <c r="AD8" s="30"/>
+      <c r="AE8" s="30"/>
+      <c r="AF8" s="71"/>
       <c r="AG8" s="65" t="s">
         <v>8</v>
       </c>
@@ -2934,9 +2926,7 @@
       </c>
     </row>
     <row r="46" spans="1:33" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="74" t="s">
-        <v>19</v>
-      </c>
+      <c r="A46" s="74"/>
       <c r="B46" s="74"/>
       <c r="C46" s="74"/>
       <c r="D46" s="74"/>

</xml_diff>